<commit_message>
Sync five hardened Alder Ridge tasks
</commit_message>
<xml_diff>
--- a/companies/alder-ridge/source-files/Shared/Finance/Reporting/2026/06 June/Q2 management reporting data book - v5 CFO scratch.xlsx
+++ b/companies/alder-ridge/source-files/Shared/Finance/Reporting/2026/06 June/Q2 management reporting data book - v5 CFO scratch.xlsx
@@ -9,8 +9,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Checks" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Quarterly KPIs'!$A$4:$M$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Board Performance'!$A$4:$M$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Quarterly KPIs'!$A$4:$M$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Board Performance'!$A$4:$M$100</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -642,7 +642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1314,7 +1314,7 @@
     <row r="15">
       <c r="A15" s="36" t="inlineStr">
         <is>
-          <t>RPT-00320</t>
+          <t>RPT-00366</t>
         </is>
       </c>
       <c r="B15" s="27" t="inlineStr">
@@ -1371,7 +1371,7 @@
     <row r="16">
       <c r="A16" s="36" t="inlineStr">
         <is>
-          <t>RPT-00321</t>
+          <t>RPT-00367</t>
         </is>
       </c>
       <c r="B16" s="27" t="inlineStr">
@@ -1428,7 +1428,7 @@
     <row r="17">
       <c r="A17" s="36" t="inlineStr">
         <is>
-          <t>RPT-00322</t>
+          <t>RPT-00368</t>
         </is>
       </c>
       <c r="B17" s="27" t="inlineStr">
@@ -1485,7 +1485,7 @@
     <row r="18">
       <c r="A18" s="36" t="inlineStr">
         <is>
-          <t>RPT-00323</t>
+          <t>RPT-00369</t>
         </is>
       </c>
       <c r="B18" s="27" t="inlineStr">
@@ -1542,7 +1542,7 @@
     <row r="19">
       <c r="A19" s="36" t="inlineStr">
         <is>
-          <t>RPT-00324</t>
+          <t>RPT-00370</t>
         </is>
       </c>
       <c r="B19" s="27" t="inlineStr">
@@ -1599,7 +1599,7 @@
     <row r="20">
       <c r="A20" s="36" t="inlineStr">
         <is>
-          <t>RPT-00325</t>
+          <t>RPT-00371</t>
         </is>
       </c>
       <c r="B20" s="27" t="inlineStr">
@@ -1656,7 +1656,7 @@
     <row r="21">
       <c r="A21" s="36" t="inlineStr">
         <is>
-          <t>RPT-00326</t>
+          <t>RPT-00372</t>
         </is>
       </c>
       <c r="B21" s="27" t="inlineStr">
@@ -1713,7 +1713,7 @@
     <row r="22">
       <c r="A22" s="36" t="inlineStr">
         <is>
-          <t>RPT-00327</t>
+          <t>RPT-00373</t>
         </is>
       </c>
       <c r="B22" s="27" t="inlineStr">
@@ -1770,7 +1770,7 @@
     <row r="23">
       <c r="A23" s="36" t="inlineStr">
         <is>
-          <t>RPT-00328</t>
+          <t>RPT-00374</t>
         </is>
       </c>
       <c r="B23" s="27" t="inlineStr">
@@ -1827,7 +1827,7 @@
     <row r="24">
       <c r="A24" s="36" t="inlineStr">
         <is>
-          <t>RPT-00329</t>
+          <t>RPT-00375</t>
         </is>
       </c>
       <c r="B24" s="27" t="inlineStr">
@@ -1884,7 +1884,7 @@
     <row r="25">
       <c r="A25" s="36" t="inlineStr">
         <is>
-          <t>RPT-00330</t>
+          <t>RPT-00376</t>
         </is>
       </c>
       <c r="B25" s="27" t="inlineStr">
@@ -1941,7 +1941,7 @@
     <row r="26">
       <c r="A26" s="36" t="inlineStr">
         <is>
-          <t>RPT-00331</t>
+          <t>RPT-00377</t>
         </is>
       </c>
       <c r="B26" s="27" t="inlineStr">
@@ -1998,7 +1998,7 @@
     <row r="27">
       <c r="A27" s="36" t="inlineStr">
         <is>
-          <t>RPT-00343</t>
+          <t>RPT-00389</t>
         </is>
       </c>
       <c r="B27" s="27" t="inlineStr">
@@ -2055,7 +2055,7 @@
     <row r="28">
       <c r="A28" s="36" t="inlineStr">
         <is>
-          <t>RPT-00344</t>
+          <t>RPT-00390</t>
         </is>
       </c>
       <c r="B28" s="27" t="inlineStr">
@@ -2112,7 +2112,7 @@
     <row r="29">
       <c r="A29" s="36" t="inlineStr">
         <is>
-          <t>RPT-00345</t>
+          <t>RPT-00391</t>
         </is>
       </c>
       <c r="B29" s="27" t="inlineStr">
@@ -2169,7 +2169,7 @@
     <row r="30">
       <c r="A30" s="36" t="inlineStr">
         <is>
-          <t>RPT-00346</t>
+          <t>RPT-00392</t>
         </is>
       </c>
       <c r="B30" s="27" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <row r="31">
       <c r="A31" s="36" t="inlineStr">
         <is>
-          <t>RPT-00347</t>
+          <t>RPT-00393</t>
         </is>
       </c>
       <c r="B31" s="27" t="inlineStr">
@@ -2283,7 +2283,7 @@
     <row r="32">
       <c r="A32" s="36" t="inlineStr">
         <is>
-          <t>RPT-00348</t>
+          <t>RPT-00394</t>
         </is>
       </c>
       <c r="B32" s="27" t="inlineStr">
@@ -2337,8 +2337,464 @@
       </c>
       <c r="M32" s="27" t="inlineStr"/>
     </row>
+    <row r="33">
+      <c r="A33" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00399</t>
+        </is>
+      </c>
+      <c r="B33" s="27" t="inlineStr">
+        <is>
+          <t>Create the restated investor KPI fact sheet</t>
+        </is>
+      </c>
+      <c r="C33" s="27" t="inlineStr">
+        <is>
+          <t>Investor KPI pending scope review</t>
+        </is>
+      </c>
+      <c r="D33" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E33" s="27" t="inlineStr">
+        <is>
+          <t>2026-05 working copy</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="inlineStr">
+        <is>
+          <t>Approved case</t>
+        </is>
+      </c>
+      <c r="G33" s="27" t="inlineStr">
+        <is>
+          <t>Pending acquired revenue exclusion</t>
+        </is>
+      </c>
+      <c r="H33" s="44" t="n">
+        <v>350200</v>
+      </c>
+      <c r="I33" s="27" t="inlineStr"/>
+      <c r="J33" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K33" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L33" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M33" s="27" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00400</t>
+        </is>
+      </c>
+      <c r="B34" s="27" t="inlineStr">
+        <is>
+          <t>Create the restated investor KPI fact sheet</t>
+        </is>
+      </c>
+      <c r="C34" s="27" t="inlineStr">
+        <is>
+          <t>Investor KPI pending scope review</t>
+        </is>
+      </c>
+      <c r="D34" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E34" s="27" t="inlineStr">
+        <is>
+          <t>Management review</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="inlineStr">
+        <is>
+          <t>Management stretch</t>
+        </is>
+      </c>
+      <c r="G34" s="27" t="inlineStr">
+        <is>
+          <t>Additional restricted cash exclusion</t>
+        </is>
+      </c>
+      <c r="H34" s="44" t="n">
+        <v>104000</v>
+      </c>
+      <c r="I34" s="27" t="inlineStr"/>
+      <c r="J34" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K34" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L34" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M34" s="27" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00401</t>
+        </is>
+      </c>
+      <c r="B35" s="27" t="inlineStr">
+        <is>
+          <t>Create the restated investor KPI fact sheet</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="inlineStr">
+        <is>
+          <t>Investor KPI pending scope review</t>
+        </is>
+      </c>
+      <c r="D35" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E35" s="27" t="inlineStr">
+        <is>
+          <t>2026-05 working copy</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="inlineStr">
+        <is>
+          <t>Approved case</t>
+        </is>
+      </c>
+      <c r="G35" s="27" t="inlineStr">
+        <is>
+          <t>Pending adjusted EBITDA reduction</t>
+        </is>
+      </c>
+      <c r="H35" s="44" t="n">
+        <v>189000</v>
+      </c>
+      <c r="I35" s="27" t="inlineStr"/>
+      <c r="J35" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K35" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L35" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M35" s="27" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00402</t>
+        </is>
+      </c>
+      <c r="B36" s="27" t="inlineStr">
+        <is>
+          <t>Create the restated investor KPI fact sheet</t>
+        </is>
+      </c>
+      <c r="C36" s="27" t="inlineStr">
+        <is>
+          <t>Investor KPI pending scope review</t>
+        </is>
+      </c>
+      <c r="D36" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E36" s="27" t="inlineStr">
+        <is>
+          <t>Management review</t>
+        </is>
+      </c>
+      <c r="F36" s="27" t="inlineStr">
+        <is>
+          <t>Management stretch</t>
+        </is>
+      </c>
+      <c r="G36" s="27" t="inlineStr">
+        <is>
+          <t>Pending disposed revenue addback</t>
+        </is>
+      </c>
+      <c r="H36" s="44" t="n">
+        <v>92.7</v>
+      </c>
+      <c r="I36" s="27" t="inlineStr"/>
+      <c r="J36" s="27" t="inlineStr">
+        <is>
+          <t>USD thousands</t>
+        </is>
+      </c>
+      <c r="K36" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L36" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M36" s="27" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00403</t>
+        </is>
+      </c>
+      <c r="B37" s="27" t="inlineStr">
+        <is>
+          <t>Create the restated investor KPI fact sheet</t>
+        </is>
+      </c>
+      <c r="C37" s="27" t="inlineStr">
+        <is>
+          <t>Investor KPI pending scope review</t>
+        </is>
+      </c>
+      <c r="D37" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E37" s="27" t="inlineStr">
+        <is>
+          <t>2026-05 working copy</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="inlineStr">
+        <is>
+          <t>Approved case</t>
+        </is>
+      </c>
+      <c r="G37" s="27" t="inlineStr">
+        <is>
+          <t>Pending acquired revenue exclusion</t>
+        </is>
+      </c>
+      <c r="H37" s="44" t="n">
+        <v>353600</v>
+      </c>
+      <c r="I37" s="27" t="inlineStr"/>
+      <c r="J37" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K37" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L37" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M37" s="27" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00404</t>
+        </is>
+      </c>
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>Create the restated investor KPI fact sheet</t>
+        </is>
+      </c>
+      <c r="C38" s="27" t="inlineStr">
+        <is>
+          <t>Investor KPI pending scope review</t>
+        </is>
+      </c>
+      <c r="D38" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E38" s="27" t="inlineStr">
+        <is>
+          <t>Management review</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="inlineStr">
+        <is>
+          <t>Management stretch</t>
+        </is>
+      </c>
+      <c r="G38" s="27" t="inlineStr">
+        <is>
+          <t>Additional restricted cash exclusion</t>
+        </is>
+      </c>
+      <c r="H38" s="44" t="n">
+        <v>105000</v>
+      </c>
+      <c r="I38" s="27" t="inlineStr"/>
+      <c r="J38" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K38" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L38" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M38" s="27" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00405</t>
+        </is>
+      </c>
+      <c r="B39" s="27" t="inlineStr">
+        <is>
+          <t>Create the restated investor KPI fact sheet</t>
+        </is>
+      </c>
+      <c r="C39" s="27" t="inlineStr">
+        <is>
+          <t>Investor KPI pending scope review</t>
+        </is>
+      </c>
+      <c r="D39" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E39" s="27" t="inlineStr">
+        <is>
+          <t>2026-05 working copy</t>
+        </is>
+      </c>
+      <c r="F39" s="27" t="inlineStr">
+        <is>
+          <t>Approved case</t>
+        </is>
+      </c>
+      <c r="G39" s="27" t="inlineStr">
+        <is>
+          <t>Pending adjusted EBITDA reduction</t>
+        </is>
+      </c>
+      <c r="H39" s="44" t="n">
+        <v>185400</v>
+      </c>
+      <c r="I39" s="27" t="inlineStr"/>
+      <c r="J39" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K39" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L39" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M39" s="27" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00406</t>
+        </is>
+      </c>
+      <c r="B40" s="27" t="inlineStr">
+        <is>
+          <t>Create the restated investor KPI fact sheet</t>
+        </is>
+      </c>
+      <c r="C40" s="27" t="inlineStr">
+        <is>
+          <t>Investor KPI pending scope review</t>
+        </is>
+      </c>
+      <c r="D40" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E40" s="27" t="inlineStr">
+        <is>
+          <t>Management review</t>
+        </is>
+      </c>
+      <c r="F40" s="27" t="inlineStr">
+        <is>
+          <t>Management stretch</t>
+        </is>
+      </c>
+      <c r="G40" s="27" t="inlineStr">
+        <is>
+          <t>Pending disposed revenue addback</t>
+        </is>
+      </c>
+      <c r="H40" s="44" t="n">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="I40" s="27" t="inlineStr"/>
+      <c r="J40" s="27" t="inlineStr">
+        <is>
+          <t>USD thousands</t>
+        </is>
+      </c>
+      <c r="K40" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L40" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M40" s="27" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M32"/>
+  <autoFilter ref="A4:M40"/>
   <mergeCells count="2">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>
@@ -2353,7 +2809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M82"/>
+  <dimension ref="A1:M100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2569,7 +3025,7 @@
     <row r="7">
       <c r="A7" s="36" t="inlineStr">
         <is>
-          <t>RPT-00094</t>
+          <t>RPT-00122</t>
         </is>
       </c>
       <c r="B7" s="27" t="inlineStr">
@@ -2626,7 +3082,7 @@
     <row r="8">
       <c r="A8" s="36" t="inlineStr">
         <is>
-          <t>RPT-00095</t>
+          <t>RPT-00123</t>
         </is>
       </c>
       <c r="B8" s="27" t="inlineStr">
@@ -2683,7 +3139,7 @@
     <row r="9">
       <c r="A9" s="36" t="inlineStr">
         <is>
-          <t>RPT-00096</t>
+          <t>RPT-00124</t>
         </is>
       </c>
       <c r="B9" s="27" t="inlineStr">
@@ -2740,7 +3196,7 @@
     <row r="10">
       <c r="A10" s="36" t="inlineStr">
         <is>
-          <t>RPT-00097</t>
+          <t>RPT-00125</t>
         </is>
       </c>
       <c r="B10" s="27" t="inlineStr">
@@ -2797,7 +3253,7 @@
     <row r="11">
       <c r="A11" s="36" t="inlineStr">
         <is>
-          <t>RPT-00098</t>
+          <t>RPT-00126</t>
         </is>
       </c>
       <c r="B11" s="27" t="inlineStr">
@@ -2854,7 +3310,7 @@
     <row r="12">
       <c r="A12" s="36" t="inlineStr">
         <is>
-          <t>RPT-00099</t>
+          <t>RPT-00127</t>
         </is>
       </c>
       <c r="B12" s="27" t="inlineStr">
@@ -2911,7 +3367,7 @@
     <row r="13">
       <c r="A13" s="36" t="inlineStr">
         <is>
-          <t>RPT-00100</t>
+          <t>RPT-00128</t>
         </is>
       </c>
       <c r="B13" s="27" t="inlineStr">
@@ -2968,7 +3424,7 @@
     <row r="14">
       <c r="A14" s="36" t="inlineStr">
         <is>
-          <t>RPT-00101</t>
+          <t>RPT-00129</t>
         </is>
       </c>
       <c r="B14" s="27" t="inlineStr">
@@ -2978,17 +3434,17 @@
       </c>
       <c r="C14" s="27" t="inlineStr">
         <is>
-          <t>Q2 approved plan</t>
+          <t>Board recovery action register</t>
         </is>
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>Construction</t>
+          <t>Collections timing</t>
         </is>
       </c>
       <c r="E14" s="27" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-Q2</t>
         </is>
       </c>
       <c r="F14" s="27" t="inlineStr">
@@ -2998,11 +3454,11 @@
       </c>
       <c r="G14" s="27" t="inlineStr">
         <is>
-          <t>EBITDA plan margin</t>
+          <t>Approved realization probability</t>
         </is>
       </c>
       <c r="H14" s="44" t="n">
-        <v>0.1196</v>
+        <v>0.8320000000000001</v>
       </c>
       <c r="I14" s="27" t="inlineStr"/>
       <c r="J14" s="27" t="inlineStr">
@@ -3025,7 +3481,7 @@
     <row r="15">
       <c r="A15" s="36" t="inlineStr">
         <is>
-          <t>RPT-00102</t>
+          <t>RPT-00130</t>
         </is>
       </c>
       <c r="B15" s="27" t="inlineStr">
@@ -3035,12 +3491,12 @@
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>Q2 actual export</t>
+          <t>Q2 approved plan</t>
         </is>
       </c>
       <c r="D15" s="27" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Construction</t>
         </is>
       </c>
       <c r="E15" s="27" t="inlineStr">
@@ -3055,16 +3511,16 @@
       </c>
       <c r="G15" s="27" t="inlineStr">
         <is>
-          <t>Adjusted EBITDA margin</t>
+          <t>Revenue plan</t>
         </is>
       </c>
       <c r="H15" s="44" t="n">
-        <v>0.1806</v>
+        <v>2507232</v>
       </c>
       <c r="I15" s="27" t="inlineStr"/>
       <c r="J15" s="27" t="inlineStr">
         <is>
-          <t>decimal ratio</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K15" s="27" t="inlineStr">
@@ -3082,7 +3538,7 @@
     <row r="16">
       <c r="A16" s="36" t="inlineStr">
         <is>
-          <t>RPT-00103</t>
+          <t>RPT-00131</t>
         </is>
       </c>
       <c r="B16" s="27" t="inlineStr">
@@ -3097,7 +3553,7 @@
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>Controls</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="E16" s="27" t="inlineStr">
@@ -3112,16 +3568,16 @@
       </c>
       <c r="G16" s="27" t="inlineStr">
         <is>
-          <t>Revenue plan</t>
+          <t>EBITDA plan margin</t>
         </is>
       </c>
       <c r="H16" s="44" t="n">
-        <v>675680</v>
+        <v>0.18334</v>
       </c>
       <c r="I16" s="27" t="inlineStr"/>
       <c r="J16" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>decimal ratio</t>
         </is>
       </c>
       <c r="K16" s="27" t="inlineStr">
@@ -3139,7 +3595,7 @@
     <row r="17">
       <c r="A17" s="36" t="inlineStr">
         <is>
-          <t>RPT-00149</t>
+          <t>RPT-00177</t>
         </is>
       </c>
       <c r="B17" s="27" t="inlineStr">
@@ -3196,7 +3652,7 @@
     <row r="18">
       <c r="A18" s="36" t="inlineStr">
         <is>
-          <t>RPT-00150</t>
+          <t>RPT-00178</t>
         </is>
       </c>
       <c r="B18" s="27" t="inlineStr">
@@ -3253,7 +3709,7 @@
     <row r="19">
       <c r="A19" s="36" t="inlineStr">
         <is>
-          <t>RPT-00157</t>
+          <t>RPT-00187</t>
         </is>
       </c>
       <c r="B19" s="27" t="inlineStr">
@@ -3310,7 +3766,7 @@
     <row r="20">
       <c r="A20" s="36" t="inlineStr">
         <is>
-          <t>RPT-00158</t>
+          <t>RPT-00188</t>
         </is>
       </c>
       <c r="B20" s="27" t="inlineStr">
@@ -3367,7 +3823,7 @@
     <row r="21">
       <c r="A21" s="36" t="inlineStr">
         <is>
-          <t>RPT-00159</t>
+          <t>RPT-00189</t>
         </is>
       </c>
       <c r="B21" s="27" t="inlineStr">
@@ -3424,7 +3880,7 @@
     <row r="22">
       <c r="A22" s="36" t="inlineStr">
         <is>
-          <t>RPT-00160</t>
+          <t>RPT-00190</t>
         </is>
       </c>
       <c r="B22" s="27" t="inlineStr">
@@ -3481,7 +3937,7 @@
     <row r="23">
       <c r="A23" s="36" t="inlineStr">
         <is>
-          <t>RPT-00161</t>
+          <t>RPT-00191</t>
         </is>
       </c>
       <c r="B23" s="27" t="inlineStr">
@@ -3515,12 +3971,12 @@
         </is>
       </c>
       <c r="H23" s="44" t="n">
-        <v>540800</v>
+        <v>540.8</v>
       </c>
       <c r="I23" s="27" t="inlineStr"/>
       <c r="J23" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>USD thousands</t>
         </is>
       </c>
       <c r="K23" s="27" t="inlineStr">
@@ -3538,7 +3994,7 @@
     <row r="24">
       <c r="A24" s="36" t="inlineStr">
         <is>
-          <t>RPT-00162</t>
+          <t>RPT-00192</t>
         </is>
       </c>
       <c r="B24" s="27" t="inlineStr">
@@ -3595,7 +4051,7 @@
     <row r="25">
       <c r="A25" s="36" t="inlineStr">
         <is>
-          <t>RPT-00163</t>
+          <t>RPT-00193</t>
         </is>
       </c>
       <c r="B25" s="27" t="inlineStr">
@@ -3629,12 +4085,12 @@
         </is>
       </c>
       <c r="H25" s="44" t="n">
-        <v>97.84999999999999</v>
+        <v>97850</v>
       </c>
       <c r="I25" s="27" t="inlineStr"/>
       <c r="J25" s="27" t="inlineStr">
         <is>
-          <t>USD thousands</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K25" s="27" t="inlineStr">
@@ -3652,7 +4108,7 @@
     <row r="26">
       <c r="A26" s="36" t="inlineStr">
         <is>
-          <t>RPT-00164</t>
+          <t>RPT-00194</t>
         </is>
       </c>
       <c r="B26" s="27" t="inlineStr">
@@ -3662,7 +4118,7 @@
       </c>
       <c r="C26" s="27" t="inlineStr">
         <is>
-          <t>Q2 approved plan</t>
+          <t>Q2 actual export</t>
         </is>
       </c>
       <c r="D26" s="27" t="inlineStr">
@@ -3682,11 +4138,11 @@
       </c>
       <c r="G26" s="27" t="inlineStr">
         <is>
-          <t>EBITDA plan margin</t>
+          <t>Adjusted EBITDA margin</t>
         </is>
       </c>
       <c r="H26" s="44" t="n">
-        <v>0.1196</v>
+        <v>0.10296</v>
       </c>
       <c r="I26" s="27" t="inlineStr"/>
       <c r="J26" s="27" t="inlineStr">
@@ -3709,7 +4165,7 @@
     <row r="27">
       <c r="A27" s="36" t="inlineStr">
         <is>
-          <t>RPT-00165</t>
+          <t>RPT-00195</t>
         </is>
       </c>
       <c r="B27" s="27" t="inlineStr">
@@ -3719,7 +4175,7 @@
       </c>
       <c r="C27" s="27" t="inlineStr">
         <is>
-          <t>Q2 actual export</t>
+          <t>Q2 approved plan</t>
         </is>
       </c>
       <c r="D27" s="27" t="inlineStr">
@@ -3739,16 +4195,16 @@
       </c>
       <c r="G27" s="27" t="inlineStr">
         <is>
-          <t>Adjusted EBITDA margin</t>
+          <t>Revenue plan</t>
         </is>
       </c>
       <c r="H27" s="44" t="n">
-        <v>0.1806</v>
+        <v>1205.4</v>
       </c>
       <c r="I27" s="27" t="inlineStr"/>
       <c r="J27" s="27" t="inlineStr">
         <is>
-          <t>decimal ratio</t>
+          <t>USD thousands</t>
         </is>
       </c>
       <c r="K27" s="27" t="inlineStr">
@@ -3766,7 +4222,7 @@
     <row r="28">
       <c r="A28" s="36" t="inlineStr">
         <is>
-          <t>RPT-00166</t>
+          <t>RPT-00196</t>
         </is>
       </c>
       <c r="B28" s="27" t="inlineStr">
@@ -3781,12 +4237,12 @@
       </c>
       <c r="D28" s="27" t="inlineStr">
         <is>
-          <t>Controls</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="E28" s="27" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F28" s="27" t="inlineStr">
@@ -3796,16 +4252,16 @@
       </c>
       <c r="G28" s="27" t="inlineStr">
         <is>
-          <t>Revenue plan</t>
+          <t>EBITDA plan margin</t>
         </is>
       </c>
       <c r="H28" s="44" t="n">
-        <v>675680</v>
+        <v>0.18334</v>
       </c>
       <c r="I28" s="27" t="inlineStr"/>
       <c r="J28" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>decimal ratio</t>
         </is>
       </c>
       <c r="K28" s="27" t="inlineStr">
@@ -3823,7 +4279,7 @@
     <row r="29">
       <c r="A29" s="36" t="inlineStr">
         <is>
-          <t>RPT-00212</t>
+          <t>RPT-00258</t>
         </is>
       </c>
       <c r="B29" s="27" t="inlineStr">
@@ -3880,7 +4336,7 @@
     <row r="30">
       <c r="A30" s="36" t="inlineStr">
         <is>
-          <t>RPT-00213</t>
+          <t>RPT-00259</t>
         </is>
       </c>
       <c r="B30" s="27" t="inlineStr">
@@ -3937,7 +4393,7 @@
     <row r="31">
       <c r="A31" s="36" t="inlineStr">
         <is>
-          <t>RPT-00222</t>
+          <t>RPT-00268</t>
         </is>
       </c>
       <c r="B31" s="27" t="inlineStr">
@@ -3994,7 +4450,7 @@
     <row r="32">
       <c r="A32" s="36" t="inlineStr">
         <is>
-          <t>RPT-00223</t>
+          <t>RPT-00269</t>
         </is>
       </c>
       <c r="B32" s="27" t="inlineStr">
@@ -4051,7 +4507,7 @@
     <row r="33">
       <c r="A33" s="36" t="inlineStr">
         <is>
-          <t>RPT-00224</t>
+          <t>RPT-00270</t>
         </is>
       </c>
       <c r="B33" s="27" t="inlineStr">
@@ -4108,7 +4564,7 @@
     <row r="34">
       <c r="A34" s="36" t="inlineStr">
         <is>
-          <t>RPT-00225</t>
+          <t>RPT-00271</t>
         </is>
       </c>
       <c r="B34" s="27" t="inlineStr">
@@ -4165,7 +4621,7 @@
     <row r="35">
       <c r="A35" s="36" t="inlineStr">
         <is>
-          <t>RPT-00226</t>
+          <t>RPT-00272</t>
         </is>
       </c>
       <c r="B35" s="27" t="inlineStr">
@@ -4222,7 +4678,7 @@
     <row r="36">
       <c r="A36" s="36" t="inlineStr">
         <is>
-          <t>RPT-00227</t>
+          <t>RPT-00273</t>
         </is>
       </c>
       <c r="B36" s="27" t="inlineStr">
@@ -4279,7 +4735,7 @@
     <row r="37">
       <c r="A37" s="36" t="inlineStr">
         <is>
-          <t>RPT-00228</t>
+          <t>RPT-00274</t>
         </is>
       </c>
       <c r="B37" s="27" t="inlineStr">
@@ -4336,7 +4792,7 @@
     <row r="38">
       <c r="A38" s="36" t="inlineStr">
         <is>
-          <t>RPT-00229</t>
+          <t>RPT-00275</t>
         </is>
       </c>
       <c r="B38" s="27" t="inlineStr">
@@ -4393,7 +4849,7 @@
     <row r="39">
       <c r="A39" s="36" t="inlineStr">
         <is>
-          <t>RPT-00230</t>
+          <t>RPT-00276</t>
         </is>
       </c>
       <c r="B39" s="27" t="inlineStr">
@@ -4450,7 +4906,7 @@
     <row r="40">
       <c r="A40" s="36" t="inlineStr">
         <is>
-          <t>RPT-00231</t>
+          <t>RPT-00277</t>
         </is>
       </c>
       <c r="B40" s="27" t="inlineStr">
@@ -4507,7 +4963,7 @@
     <row r="41">
       <c r="A41" s="36" t="inlineStr">
         <is>
-          <t>RPT-00263</t>
+          <t>RPT-00309</t>
         </is>
       </c>
       <c r="B41" s="27" t="inlineStr">
@@ -4564,7 +5020,7 @@
     <row r="42">
       <c r="A42" s="36" t="inlineStr">
         <is>
-          <t>RPT-00264</t>
+          <t>RPT-00310</t>
         </is>
       </c>
       <c r="B42" s="27" t="inlineStr">
@@ -4621,7 +5077,7 @@
     <row r="43">
       <c r="A43" s="36" t="inlineStr">
         <is>
-          <t>RPT-00265</t>
+          <t>RPT-00311</t>
         </is>
       </c>
       <c r="B43" s="27" t="inlineStr">
@@ -4678,7 +5134,7 @@
     <row r="44">
       <c r="A44" s="36" t="inlineStr">
         <is>
-          <t>RPT-00266</t>
+          <t>RPT-00312</t>
         </is>
       </c>
       <c r="B44" s="27" t="inlineStr">
@@ -4735,7 +5191,7 @@
     <row r="45">
       <c r="A45" s="36" t="inlineStr">
         <is>
-          <t>RPT-00267</t>
+          <t>RPT-00313</t>
         </is>
       </c>
       <c r="B45" s="27" t="inlineStr">
@@ -4792,7 +5248,7 @@
     <row r="46">
       <c r="A46" s="36" t="inlineStr">
         <is>
-          <t>RPT-00268</t>
+          <t>RPT-00314</t>
         </is>
       </c>
       <c r="B46" s="27" t="inlineStr">
@@ -4849,7 +5305,7 @@
     <row r="47">
       <c r="A47" s="36" t="inlineStr">
         <is>
-          <t>RPT-00269</t>
+          <t>RPT-00315</t>
         </is>
       </c>
       <c r="B47" s="27" t="inlineStr">
@@ -4906,7 +5362,7 @@
     <row r="48">
       <c r="A48" s="36" t="inlineStr">
         <is>
-          <t>RPT-00270</t>
+          <t>RPT-00316</t>
         </is>
       </c>
       <c r="B48" s="27" t="inlineStr">
@@ -4963,7 +5419,7 @@
     <row r="49">
       <c r="A49" s="36" t="inlineStr">
         <is>
-          <t>RPT-00271</t>
+          <t>RPT-00317</t>
         </is>
       </c>
       <c r="B49" s="27" t="inlineStr">
@@ -5020,7 +5476,7 @@
     <row r="50">
       <c r="A50" s="36" t="inlineStr">
         <is>
-          <t>RPT-00272</t>
+          <t>RPT-00318</t>
         </is>
       </c>
       <c r="B50" s="27" t="inlineStr">
@@ -5077,7 +5533,7 @@
     <row r="51">
       <c r="A51" s="36" t="inlineStr">
         <is>
-          <t>RPT-00273</t>
+          <t>RPT-00319</t>
         </is>
       </c>
       <c r="B51" s="27" t="inlineStr">
@@ -5134,7 +5590,7 @@
     <row r="52">
       <c r="A52" s="36" t="inlineStr">
         <is>
-          <t>RPT-00274</t>
+          <t>RPT-00320</t>
         </is>
       </c>
       <c r="B52" s="27" t="inlineStr">
@@ -5191,7 +5647,7 @@
     <row r="53">
       <c r="A53" s="36" t="inlineStr">
         <is>
-          <t>RPT-00275</t>
+          <t>RPT-00321</t>
         </is>
       </c>
       <c r="B53" s="27" t="inlineStr">
@@ -5248,7 +5704,7 @@
     <row r="54">
       <c r="A54" s="36" t="inlineStr">
         <is>
-          <t>RPT-00276</t>
+          <t>RPT-00322</t>
         </is>
       </c>
       <c r="B54" s="27" t="inlineStr">
@@ -5305,7 +5761,7 @@
     <row r="55">
       <c r="A55" s="36" t="inlineStr">
         <is>
-          <t>RPT-00286</t>
+          <t>RPT-00332</t>
         </is>
       </c>
       <c r="B55" s="27" t="inlineStr">
@@ -5362,7 +5818,7 @@
     <row r="56">
       <c r="A56" s="36" t="inlineStr">
         <is>
-          <t>RPT-00287</t>
+          <t>RPT-00333</t>
         </is>
       </c>
       <c r="B56" s="27" t="inlineStr">
@@ -5419,7 +5875,7 @@
     <row r="57">
       <c r="A57" s="36" t="inlineStr">
         <is>
-          <t>RPT-00288</t>
+          <t>RPT-00334</t>
         </is>
       </c>
       <c r="B57" s="27" t="inlineStr">
@@ -5476,7 +5932,7 @@
     <row r="58">
       <c r="A58" s="36" t="inlineStr">
         <is>
-          <t>RPT-00289</t>
+          <t>RPT-00335</t>
         </is>
       </c>
       <c r="B58" s="27" t="inlineStr">
@@ -5533,7 +5989,7 @@
     <row r="59">
       <c r="A59" s="36" t="inlineStr">
         <is>
-          <t>RPT-00290</t>
+          <t>RPT-00336</t>
         </is>
       </c>
       <c r="B59" s="27" t="inlineStr">
@@ -5590,7 +6046,7 @@
     <row r="60">
       <c r="A60" s="36" t="inlineStr">
         <is>
-          <t>RPT-00291</t>
+          <t>RPT-00337</t>
         </is>
       </c>
       <c r="B60" s="27" t="inlineStr">
@@ -5647,22 +6103,22 @@
     <row r="61">
       <c r="A61" s="36" t="inlineStr">
         <is>
-          <t>RPT-00393</t>
+          <t>RPT-097X37</t>
         </is>
       </c>
       <c r="B61" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C61" s="27" t="inlineStr">
         <is>
-          <t>Board operating outlook</t>
+          <t>Guidance protection action register</t>
         </is>
       </c>
       <c r="D61" s="27" t="inlineStr">
         <is>
-          <t>Construction</t>
+          <t>Copper price collar</t>
         </is>
       </c>
       <c r="E61" s="27" t="inlineStr">
@@ -5677,11 +6133,11 @@
       </c>
       <c r="G61" s="27" t="inlineStr">
         <is>
-          <t>Forecast revenue</t>
+          <t>Cash cost</t>
         </is>
       </c>
       <c r="H61" s="44" t="n">
-        <v>32393500</v>
+        <v>149350</v>
       </c>
       <c r="I61" s="27" t="inlineStr"/>
       <c r="J61" s="27" t="inlineStr">
@@ -5704,27 +6160,27 @@
     <row r="62">
       <c r="A62" s="36" t="inlineStr">
         <is>
-          <t>RPT-00394</t>
+          <t>RPT-097X38</t>
         </is>
       </c>
       <c r="B62" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C62" s="27" t="inlineStr">
         <is>
-          <t>Board operating outlook</t>
+          <t>Guidance protection action register</t>
         </is>
       </c>
       <c r="D62" s="27" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Construction buyout reset</t>
         </is>
       </c>
       <c r="E62" s="27" t="inlineStr">
         <is>
-          <t>FY26</t>
+          <t>Management review</t>
         </is>
       </c>
       <c r="F62" s="27" t="inlineStr">
@@ -5734,16 +6190,16 @@
       </c>
       <c r="G62" s="27" t="inlineStr">
         <is>
-          <t>Plan revenue</t>
+          <t>Capacity units</t>
         </is>
       </c>
       <c r="H62" s="44" t="n">
-        <v>14196000</v>
+        <v>249.6</v>
       </c>
       <c r="I62" s="27" t="inlineStr"/>
       <c r="J62" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>forecast-response points</t>
         </is>
       </c>
       <c r="K62" s="27" t="inlineStr">
@@ -5761,22 +6217,22 @@
     <row r="63">
       <c r="A63" s="36" t="inlineStr">
         <is>
-          <t>RPT-00395</t>
+          <t>RPT-097X39</t>
         </is>
       </c>
       <c r="B63" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C63" s="27" t="inlineStr">
         <is>
-          <t>Board operating outlook</t>
+          <t>Guidance protection action register</t>
         </is>
       </c>
       <c r="D63" s="27" t="inlineStr">
         <is>
-          <t>Controls</t>
+          <t>Discretionary opex hold</t>
         </is>
       </c>
       <c r="E63" s="27" t="inlineStr">
@@ -5791,11 +6247,11 @@
       </c>
       <c r="G63" s="27" t="inlineStr">
         <is>
-          <t>Forecast gross margin</t>
+          <t>Realization probability</t>
         </is>
       </c>
       <c r="H63" s="44" t="n">
-        <v>0.30975</v>
+        <v>0.9660000000000001</v>
       </c>
       <c r="I63" s="27" t="inlineStr"/>
       <c r="J63" s="27" t="inlineStr">
@@ -5818,27 +6274,27 @@
     <row r="64">
       <c r="A64" s="36" t="inlineStr">
         <is>
-          <t>RPT-00396</t>
+          <t>RPT-097X40</t>
         </is>
       </c>
       <c r="B64" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C64" s="27" t="inlineStr">
         <is>
-          <t>Board risk outlook</t>
+          <t>Guidance protection action register</t>
         </is>
       </c>
       <c r="D64" s="27" t="inlineStr">
         <is>
-          <t>Alder Ridge</t>
+          <t>Portfolio policy</t>
         </is>
       </c>
       <c r="E64" s="27" t="inlineStr">
         <is>
-          <t>Downside</t>
+          <t>Management review</t>
         </is>
       </c>
       <c r="F64" s="27" t="inlineStr">
@@ -5848,16 +6304,16 @@
       </c>
       <c r="G64" s="27" t="inlineStr">
         <is>
-          <t>Covenant EBITDA</t>
+          <t>Capacity limit</t>
         </is>
       </c>
       <c r="H64" s="44" t="n">
-        <v>3893.4</v>
+        <v>968.2</v>
       </c>
       <c r="I64" s="27" t="inlineStr"/>
       <c r="J64" s="27" t="inlineStr">
         <is>
-          <t>USD thousands</t>
+          <t>forecast-response points</t>
         </is>
       </c>
       <c r="K64" s="27" t="inlineStr">
@@ -5875,22 +6331,22 @@
     <row r="65">
       <c r="A65" s="36" t="inlineStr">
         <is>
-          <t>RPT-00397</t>
+          <t>RPT-097X41</t>
         </is>
       </c>
       <c r="B65" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C65" s="27" t="inlineStr">
         <is>
-          <t>Board strategic priorities</t>
+          <t>Guidance protection action register</t>
         </is>
       </c>
       <c r="D65" s="27" t="inlineStr">
         <is>
-          <t>Procurement program</t>
+          <t>Construction buyout reset</t>
         </is>
       </c>
       <c r="E65" s="27" t="inlineStr">
@@ -5905,16 +6361,16 @@
       </c>
       <c r="G65" s="27" t="inlineStr">
         <is>
-          <t>Realization probability</t>
+          <t>Cash cost</t>
         </is>
       </c>
       <c r="H65" s="44" t="n">
-        <v>0.8320000000000001</v>
+        <v>140400</v>
       </c>
       <c r="I65" s="27" t="inlineStr"/>
       <c r="J65" s="27" t="inlineStr">
         <is>
-          <t>decimal ratio</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K65" s="27" t="inlineStr">
@@ -5932,27 +6388,27 @@
     <row r="66">
       <c r="A66" s="36" t="inlineStr">
         <is>
-          <t>RPT-00398</t>
+          <t>RPT-097X42</t>
         </is>
       </c>
       <c r="B66" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C66" s="27" t="inlineStr">
         <is>
-          <t>Board presentation controls</t>
+          <t>Guidance protection action register</t>
         </is>
       </c>
       <c r="D66" s="27" t="inlineStr">
         <is>
-          <t>Alder Ridge</t>
+          <t>Service labor recovery</t>
         </is>
       </c>
       <c r="E66" s="27" t="inlineStr">
         <is>
-          <t>FY26</t>
+          <t>Management review</t>
         </is>
       </c>
       <c r="F66" s="27" t="inlineStr">
@@ -5962,16 +6418,16 @@
       </c>
       <c r="G66" s="27" t="inlineStr">
         <is>
-          <t>Minimum cash</t>
+          <t>Capacity units</t>
         </is>
       </c>
       <c r="H66" s="44" t="n">
-        <v>2362500</v>
+        <v>231</v>
       </c>
       <c r="I66" s="27" t="inlineStr"/>
       <c r="J66" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>forecast-response points</t>
         </is>
       </c>
       <c r="K66" s="27" t="inlineStr">
@@ -5989,22 +6445,22 @@
     <row r="67">
       <c r="A67" s="36" t="inlineStr">
         <is>
-          <t>RPT-00399</t>
+          <t>RPT-097X43</t>
         </is>
       </c>
       <c r="B67" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C67" s="27" t="inlineStr">
         <is>
-          <t>Board operating outlook</t>
+          <t>Guidance protection action register</t>
         </is>
       </c>
       <c r="D67" s="27" t="inlineStr">
         <is>
-          <t>Construction</t>
+          <t>Backlog acceleration program</t>
         </is>
       </c>
       <c r="E67" s="27" t="inlineStr">
@@ -6019,11 +6475,11 @@
       </c>
       <c r="G67" s="27" t="inlineStr">
         <is>
-          <t>Forecast gross margin</t>
+          <t>Realization probability</t>
         </is>
       </c>
       <c r="H67" s="44" t="n">
-        <v>0.23896</v>
+        <v>0.6386000000000001</v>
       </c>
       <c r="I67" s="27" t="inlineStr"/>
       <c r="J67" s="27" t="inlineStr">
@@ -6046,27 +6502,27 @@
     <row r="68">
       <c r="A68" s="36" t="inlineStr">
         <is>
-          <t>RPT-00400</t>
+          <t>RPT-097X44</t>
         </is>
       </c>
       <c r="B68" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C68" s="27" t="inlineStr">
         <is>
-          <t>Board operating outlook</t>
+          <t>Guidance protection action register</t>
         </is>
       </c>
       <c r="D68" s="27" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Copper price collar</t>
         </is>
       </c>
       <c r="E68" s="27" t="inlineStr">
         <is>
-          <t>FY26</t>
+          <t>Management review</t>
         </is>
       </c>
       <c r="F68" s="27" t="inlineStr">
@@ -6076,16 +6532,16 @@
       </c>
       <c r="G68" s="27" t="inlineStr">
         <is>
-          <t>Plan gross margin</t>
+          <t>Gross financial effect</t>
         </is>
       </c>
       <c r="H68" s="44" t="n">
-        <v>0.442</v>
+        <v>540.8</v>
       </c>
       <c r="I68" s="27" t="inlineStr"/>
       <c r="J68" s="27" t="inlineStr">
         <is>
-          <t>decimal ratio</t>
+          <t>USD thousands</t>
         </is>
       </c>
       <c r="K68" s="27" t="inlineStr">
@@ -6103,22 +6559,22 @@
     <row r="69">
       <c r="A69" s="36" t="inlineStr">
         <is>
-          <t>RPT-00401</t>
+          <t>RPT-097X45</t>
         </is>
       </c>
       <c r="B69" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C69" s="27" t="inlineStr">
         <is>
-          <t>Board operating outlook</t>
+          <t>Guidance protection action register</t>
         </is>
       </c>
       <c r="D69" s="27" t="inlineStr">
         <is>
-          <t>Controls</t>
+          <t>Service labor recovery</t>
         </is>
       </c>
       <c r="E69" s="27" t="inlineStr">
@@ -6133,11 +6589,11 @@
       </c>
       <c r="G69" s="27" t="inlineStr">
         <is>
-          <t>Forecast opex</t>
+          <t>Cash cost</t>
         </is>
       </c>
       <c r="H69" s="44" t="n">
-        <v>1113000</v>
+        <v>126000</v>
       </c>
       <c r="I69" s="27" t="inlineStr"/>
       <c r="J69" s="27" t="inlineStr">
@@ -6160,27 +6616,27 @@
     <row r="70">
       <c r="A70" s="36" t="inlineStr">
         <is>
-          <t>RPT-00402</t>
+          <t>RPT-097X46</t>
         </is>
       </c>
       <c r="B70" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C70" s="27" t="inlineStr">
         <is>
-          <t>Board risk outlook</t>
+          <t>Guidance protection action register</t>
         </is>
       </c>
       <c r="D70" s="27" t="inlineStr">
         <is>
-          <t>Alder Ridge</t>
+          <t>Discretionary opex hold</t>
         </is>
       </c>
       <c r="E70" s="27" t="inlineStr">
         <is>
-          <t>Downside</t>
+          <t>Management review</t>
         </is>
       </c>
       <c r="F70" s="27" t="inlineStr">
@@ -6190,16 +6646,16 @@
       </c>
       <c r="G70" s="27" t="inlineStr">
         <is>
-          <t>Revolver balance</t>
+          <t>Capacity units</t>
         </is>
       </c>
       <c r="H70" s="44" t="n">
-        <v>4738000</v>
+        <v>175.1</v>
       </c>
       <c r="I70" s="27" t="inlineStr"/>
       <c r="J70" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>forecast-response points</t>
         </is>
       </c>
       <c r="K70" s="27" t="inlineStr">
@@ -6217,22 +6673,22 @@
     <row r="71">
       <c r="A71" s="36" t="inlineStr">
         <is>
-          <t>RPT-00403</t>
+          <t>RPT-097X87</t>
         </is>
       </c>
       <c r="B71" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C71" s="27" t="inlineStr">
         <is>
-          <t>Board strategic priorities</t>
+          <t>Guidance protection action register scenario controls</t>
         </is>
       </c>
       <c r="D71" s="27" t="inlineStr">
         <is>
-          <t>Service technician hiring</t>
+          <t>Board guidance base</t>
         </is>
       </c>
       <c r="E71" s="27" t="inlineStr">
@@ -6247,11 +6703,11 @@
       </c>
       <c r="G71" s="27" t="inlineStr">
         <is>
-          <t>Realization probability</t>
+          <t>Gross effect factor</t>
         </is>
       </c>
       <c r="H71" s="44" t="n">
-        <v>0.728</v>
+        <v>1.03</v>
       </c>
       <c r="I71" s="27" t="inlineStr"/>
       <c r="J71" s="27" t="inlineStr">
@@ -6274,27 +6730,27 @@
     <row r="72">
       <c r="A72" s="36" t="inlineStr">
         <is>
-          <t>RPT-00404</t>
+          <t>RPT-097X88</t>
         </is>
       </c>
       <c r="B72" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C72" s="27" t="inlineStr">
         <is>
-          <t>Board presentation controls</t>
+          <t>Guidance protection action register scenario controls</t>
         </is>
       </c>
       <c r="D72" s="27" t="inlineStr">
         <is>
-          <t>Alder Ridge</t>
+          <t>Copper and buyout squeeze</t>
         </is>
       </c>
       <c r="E72" s="27" t="inlineStr">
         <is>
-          <t>FY26</t>
+          <t>Management review</t>
         </is>
       </c>
       <c r="F72" s="27" t="inlineStr">
@@ -6304,16 +6760,16 @@
       </c>
       <c r="G72" s="27" t="inlineStr">
         <is>
-          <t>Maximum leverage</t>
+          <t>Gross effect factor</t>
         </is>
       </c>
       <c r="H72" s="44" t="n">
-        <v>2.625</v>
+        <v>0.8528</v>
       </c>
       <c r="I72" s="27" t="inlineStr"/>
       <c r="J72" s="27" t="inlineStr">
         <is>
-          <t>multiple</t>
+          <t>decimal ratio</t>
         </is>
       </c>
       <c r="K72" s="27" t="inlineStr">
@@ -6331,22 +6787,22 @@
     <row r="73">
       <c r="A73" s="36" t="inlineStr">
         <is>
-          <t>RPT-00405</t>
+          <t>RPT-097X89</t>
         </is>
       </c>
       <c r="B73" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C73" s="27" t="inlineStr">
         <is>
-          <t>Board operating outlook</t>
+          <t>Guidance protection action register scenario controls</t>
         </is>
       </c>
       <c r="D73" s="27" t="inlineStr">
         <is>
-          <t>Construction</t>
+          <t>Service labor recovery delay</t>
         </is>
       </c>
       <c r="E73" s="27" t="inlineStr">
@@ -6361,16 +6817,16 @@
       </c>
       <c r="G73" s="27" t="inlineStr">
         <is>
-          <t>Forecast opex</t>
+          <t>Gross effect factor</t>
         </is>
       </c>
       <c r="H73" s="44" t="n">
-        <v>1905500</v>
+        <v>0.903</v>
       </c>
       <c r="I73" s="27" t="inlineStr"/>
       <c r="J73" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>decimal ratio</t>
         </is>
       </c>
       <c r="K73" s="27" t="inlineStr">
@@ -6388,27 +6844,27 @@
     <row r="74">
       <c r="A74" s="36" t="inlineStr">
         <is>
-          <t>RPT-00406</t>
+          <t>RPT-097X90</t>
         </is>
       </c>
       <c r="B74" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C74" s="27" t="inlineStr">
         <is>
-          <t>Board operating outlook</t>
+          <t>Guidance protection action register scenario controls</t>
         </is>
       </c>
       <c r="D74" s="27" t="inlineStr">
         <is>
-          <t>Service</t>
+          <t>Backlog conversion shortfall</t>
         </is>
       </c>
       <c r="E74" s="27" t="inlineStr">
         <is>
-          <t>FY26</t>
+          <t>Management review</t>
         </is>
       </c>
       <c r="F74" s="27" t="inlineStr">
@@ -6418,16 +6874,16 @@
       </c>
       <c r="G74" s="27" t="inlineStr">
         <is>
-          <t>Plan opex</t>
+          <t>Gross effect factor</t>
         </is>
       </c>
       <c r="H74" s="44" t="n">
-        <v>2059200</v>
+        <v>0.7416</v>
       </c>
       <c r="I74" s="27" t="inlineStr"/>
       <c r="J74" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>decimal ratio</t>
         </is>
       </c>
       <c r="K74" s="27" t="inlineStr">
@@ -6445,22 +6901,22 @@
     <row r="75">
       <c r="A75" s="36" t="inlineStr">
         <is>
-          <t>RPT-00407</t>
+          <t>RPT-097X91</t>
         </is>
       </c>
       <c r="B75" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C75" s="27" t="inlineStr">
         <is>
-          <t>Board risk outlook</t>
+          <t>Guidance protection action register scenario controls</t>
         </is>
       </c>
       <c r="D75" s="27" t="inlineStr">
         <is>
-          <t>Alder Ridge</t>
+          <t>Combined guidance downside</t>
         </is>
       </c>
       <c r="E75" s="27" t="inlineStr">
@@ -6475,16 +6931,16 @@
       </c>
       <c r="G75" s="27" t="inlineStr">
         <is>
-          <t>Covenant EBITDA</t>
+          <t>Gross effect factor</t>
         </is>
       </c>
       <c r="H75" s="44" t="n">
-        <v>5796000</v>
+        <v>0.624</v>
       </c>
       <c r="I75" s="27" t="inlineStr"/>
       <c r="J75" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>decimal ratio</t>
         </is>
       </c>
       <c r="K75" s="27" t="inlineStr">
@@ -6502,27 +6958,27 @@
     <row r="76">
       <c r="A76" s="36" t="inlineStr">
         <is>
-          <t>RPT-00408</t>
+          <t>RPT-097X92</t>
         </is>
       </c>
       <c r="B76" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C76" s="27" t="inlineStr">
         <is>
-          <t>Board risk outlook</t>
+          <t>Guidance protection action register scenario controls</t>
         </is>
       </c>
       <c r="D76" s="27" t="inlineStr">
         <is>
-          <t>Alder Ridge</t>
+          <t>Board guidance base</t>
         </is>
       </c>
       <c r="E76" s="27" t="inlineStr">
         <is>
-          <t>Severe</t>
+          <t>Management review</t>
         </is>
       </c>
       <c r="F76" s="27" t="inlineStr">
@@ -6532,16 +6988,16 @@
       </c>
       <c r="G76" s="27" t="inlineStr">
         <is>
-          <t>Ending cash before financing</t>
+          <t>Gross effect factor</t>
         </is>
       </c>
       <c r="H76" s="44" t="n">
-        <v>844.6</v>
+        <v>1.05</v>
       </c>
       <c r="I76" s="27" t="inlineStr"/>
       <c r="J76" s="27" t="inlineStr">
         <is>
-          <t>USD thousands</t>
+          <t>decimal ratio</t>
         </is>
       </c>
       <c r="K76" s="27" t="inlineStr">
@@ -6559,22 +7015,22 @@
     <row r="77">
       <c r="A77" s="36" t="inlineStr">
         <is>
-          <t>RPT-00426</t>
+          <t>RPT-097X93</t>
         </is>
       </c>
       <c r="B77" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C77" s="27" t="inlineStr">
         <is>
-          <t>Board decision portfolio</t>
+          <t>Guidance protection action register scenario controls</t>
         </is>
       </c>
       <c r="D77" s="27" t="inlineStr">
         <is>
-          <t>Procurement program</t>
+          <t>Copper and buyout squeeze</t>
         </is>
       </c>
       <c r="E77" s="27" t="inlineStr">
@@ -6589,16 +7045,16 @@
       </c>
       <c r="G77" s="27" t="inlineStr">
         <is>
-          <t>Cash investment</t>
+          <t>Gross effect factor</t>
         </is>
       </c>
       <c r="H77" s="44" t="n">
-        <v>432600</v>
+        <v>0.8446</v>
       </c>
       <c r="I77" s="27" t="inlineStr"/>
       <c r="J77" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>decimal ratio</t>
         </is>
       </c>
       <c r="K77" s="27" t="inlineStr">
@@ -6616,27 +7072,27 @@
     <row r="78">
       <c r="A78" s="36" t="inlineStr">
         <is>
-          <t>RPT-00427</t>
+          <t>RPT-097X94</t>
         </is>
       </c>
       <c r="B78" s="27" t="inlineStr">
         <is>
-          <t>Create the CFO strategic-finance board deck</t>
+          <t>Earnings guidance range and probability bridge</t>
         </is>
       </c>
       <c r="C78" s="27" t="inlineStr">
         <is>
-          <t>Board decision portfolio</t>
+          <t>Guidance protection action register scenario controls</t>
         </is>
       </c>
       <c r="D78" s="27" t="inlineStr">
         <is>
-          <t>Pioneer acquisition</t>
+          <t>Service labor recovery delay</t>
         </is>
       </c>
       <c r="E78" s="27" t="inlineStr">
         <is>
-          <t>FY27</t>
+          <t>Management review</t>
         </is>
       </c>
       <c r="F78" s="27" t="inlineStr">
@@ -6646,11 +7102,11 @@
       </c>
       <c r="G78" s="27" t="inlineStr">
         <is>
-          <t>Severe benefit factor</t>
+          <t>Gross effect factor</t>
         </is>
       </c>
       <c r="H78" s="44" t="n">
-        <v>0.468</v>
+        <v>0.8944</v>
       </c>
       <c r="I78" s="27" t="inlineStr"/>
       <c r="J78" s="27" t="inlineStr">
@@ -6673,7 +7129,7 @@
     <row r="79">
       <c r="A79" s="36" t="inlineStr">
         <is>
-          <t>RPT-00428</t>
+          <t>RPT-00451</t>
         </is>
       </c>
       <c r="B79" s="27" t="inlineStr">
@@ -6683,12 +7139,12 @@
       </c>
       <c r="C79" s="27" t="inlineStr">
         <is>
-          <t>Board decision portfolio</t>
+          <t>Board operating outlook</t>
         </is>
       </c>
       <c r="D79" s="27" t="inlineStr">
         <is>
-          <t>Service technician hiring</t>
+          <t>Construction</t>
         </is>
       </c>
       <c r="E79" s="27" t="inlineStr">
@@ -6703,16 +7159,16 @@
       </c>
       <c r="G79" s="27" t="inlineStr">
         <is>
-          <t>Severe benefit factor</t>
+          <t>Forecast revenue</t>
         </is>
       </c>
       <c r="H79" s="44" t="n">
-        <v>0.6825000000000001</v>
+        <v>32393500</v>
       </c>
       <c r="I79" s="27" t="inlineStr"/>
       <c r="J79" s="27" t="inlineStr">
         <is>
-          <t>decimal ratio</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K79" s="27" t="inlineStr">
@@ -6730,7 +7186,7 @@
     <row r="80">
       <c r="A80" s="36" t="inlineStr">
         <is>
-          <t>RPT-00429</t>
+          <t>RPT-00452</t>
         </is>
       </c>
       <c r="B80" s="27" t="inlineStr">
@@ -6740,17 +7196,17 @@
       </c>
       <c r="C80" s="27" t="inlineStr">
         <is>
-          <t>Board decision portfolio policy</t>
+          <t>Board operating outlook</t>
         </is>
       </c>
       <c r="D80" s="27" t="inlineStr">
         <is>
-          <t>Alder Ridge</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="E80" s="27" t="inlineStr">
         <is>
-          <t>FY27</t>
+          <t>FY26</t>
         </is>
       </c>
       <c r="F80" s="27" t="inlineStr">
@@ -6760,16 +7216,16 @@
       </c>
       <c r="G80" s="27" t="inlineStr">
         <is>
-          <t>Severe EBITDA cash conversion</t>
+          <t>Plan revenue</t>
         </is>
       </c>
       <c r="H80" s="44" t="n">
-        <v>0.721</v>
+        <v>14196000</v>
       </c>
       <c r="I80" s="27" t="inlineStr"/>
       <c r="J80" s="27" t="inlineStr">
         <is>
-          <t>decimal ratio</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="K80" s="27" t="inlineStr">
@@ -6787,7 +7243,7 @@
     <row r="81">
       <c r="A81" s="36" t="inlineStr">
         <is>
-          <t>RPT-00430</t>
+          <t>RPT-00453</t>
         </is>
       </c>
       <c r="B81" s="27" t="inlineStr">
@@ -6797,12 +7253,12 @@
       </c>
       <c r="C81" s="27" t="inlineStr">
         <is>
-          <t>Board decision portfolio</t>
+          <t>Board operating outlook</t>
         </is>
       </c>
       <c r="D81" s="27" t="inlineStr">
         <is>
-          <t>Pioneer acquisition</t>
+          <t>Controls</t>
         </is>
       </c>
       <c r="E81" s="27" t="inlineStr">
@@ -6817,16 +7273,16 @@
       </c>
       <c r="G81" s="27" t="inlineStr">
         <is>
-          <t>Cash investment</t>
+          <t>Forecast gross margin</t>
         </is>
       </c>
       <c r="H81" s="44" t="n">
-        <v>1196000</v>
+        <v>0.30975</v>
       </c>
       <c r="I81" s="27" t="inlineStr"/>
       <c r="J81" s="27" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>decimal ratio</t>
         </is>
       </c>
       <c r="K81" s="27" t="inlineStr">
@@ -6844,7 +7300,7 @@
     <row r="82">
       <c r="A82" s="36" t="inlineStr">
         <is>
-          <t>RPT-00431</t>
+          <t>RPT-00454</t>
         </is>
       </c>
       <c r="B82" s="27" t="inlineStr">
@@ -6854,17 +7310,17 @@
       </c>
       <c r="C82" s="27" t="inlineStr">
         <is>
-          <t>Board decision portfolio</t>
+          <t>Board risk outlook</t>
         </is>
       </c>
       <c r="D82" s="27" t="inlineStr">
         <is>
-          <t>Service technician hiring</t>
+          <t>Alder Ridge</t>
         </is>
       </c>
       <c r="E82" s="27" t="inlineStr">
         <is>
-          <t>FY27</t>
+          <t>Downside</t>
         </is>
       </c>
       <c r="F82" s="27" t="inlineStr">
@@ -6874,32 +7330,1058 @@
       </c>
       <c r="G82" s="27" t="inlineStr">
         <is>
-          <t>Cash investment</t>
+          <t>Covenant EBITDA</t>
         </is>
       </c>
       <c r="H82" s="44" t="n">
-        <v>640500</v>
+        <v>3893.4</v>
       </c>
       <c r="I82" s="27" t="inlineStr"/>
       <c r="J82" s="27" t="inlineStr">
         <is>
+          <t>USD thousands</t>
+        </is>
+      </c>
+      <c r="K82" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L82" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M82" s="27" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00455</t>
+        </is>
+      </c>
+      <c r="B83" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C83" s="27" t="inlineStr">
+        <is>
+          <t>Board strategic priorities</t>
+        </is>
+      </c>
+      <c r="D83" s="27" t="inlineStr">
+        <is>
+          <t>Procurement program</t>
+        </is>
+      </c>
+      <c r="E83" s="27" t="inlineStr">
+        <is>
+          <t>2026-05 working copy</t>
+        </is>
+      </c>
+      <c r="F83" s="27" t="inlineStr">
+        <is>
+          <t>Approved case</t>
+        </is>
+      </c>
+      <c r="G83" s="27" t="inlineStr">
+        <is>
+          <t>Realization probability</t>
+        </is>
+      </c>
+      <c r="H83" s="44" t="n">
+        <v>0.8320000000000001</v>
+      </c>
+      <c r="I83" s="27" t="inlineStr"/>
+      <c r="J83" s="27" t="inlineStr">
+        <is>
+          <t>decimal ratio</t>
+        </is>
+      </c>
+      <c r="K83" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L83" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M83" s="27" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00456</t>
+        </is>
+      </c>
+      <c r="B84" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C84" s="27" t="inlineStr">
+        <is>
+          <t>Board presentation controls</t>
+        </is>
+      </c>
+      <c r="D84" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E84" s="27" t="inlineStr">
+        <is>
+          <t>FY26</t>
+        </is>
+      </c>
+      <c r="F84" s="27" t="inlineStr">
+        <is>
+          <t>Management stretch</t>
+        </is>
+      </c>
+      <c r="G84" s="27" t="inlineStr">
+        <is>
+          <t>Minimum cash</t>
+        </is>
+      </c>
+      <c r="H84" s="44" t="n">
+        <v>2362500</v>
+      </c>
+      <c r="I84" s="27" t="inlineStr"/>
+      <c r="J84" s="27" t="inlineStr">
+        <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="K82" s="27" t="inlineStr">
-        <is>
-          <t>Earlier management working export</t>
-        </is>
-      </c>
-      <c r="L82" s="45" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
-      <c r="M82" s="27" t="inlineStr"/>
+      <c r="K84" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L84" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M84" s="27" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00457</t>
+        </is>
+      </c>
+      <c r="B85" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C85" s="27" t="inlineStr">
+        <is>
+          <t>Board operating outlook</t>
+        </is>
+      </c>
+      <c r="D85" s="27" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="E85" s="27" t="inlineStr">
+        <is>
+          <t>2026-05 working copy</t>
+        </is>
+      </c>
+      <c r="F85" s="27" t="inlineStr">
+        <is>
+          <t>Approved case</t>
+        </is>
+      </c>
+      <c r="G85" s="27" t="inlineStr">
+        <is>
+          <t>Forecast gross margin</t>
+        </is>
+      </c>
+      <c r="H85" s="44" t="n">
+        <v>0.23896</v>
+      </c>
+      <c r="I85" s="27" t="inlineStr"/>
+      <c r="J85" s="27" t="inlineStr">
+        <is>
+          <t>decimal ratio</t>
+        </is>
+      </c>
+      <c r="K85" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L85" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M85" s="27" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00458</t>
+        </is>
+      </c>
+      <c r="B86" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C86" s="27" t="inlineStr">
+        <is>
+          <t>Board operating outlook</t>
+        </is>
+      </c>
+      <c r="D86" s="27" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E86" s="27" t="inlineStr">
+        <is>
+          <t>FY26</t>
+        </is>
+      </c>
+      <c r="F86" s="27" t="inlineStr">
+        <is>
+          <t>Management stretch</t>
+        </is>
+      </c>
+      <c r="G86" s="27" t="inlineStr">
+        <is>
+          <t>Plan gross margin</t>
+        </is>
+      </c>
+      <c r="H86" s="44" t="n">
+        <v>0.442</v>
+      </c>
+      <c r="I86" s="27" t="inlineStr"/>
+      <c r="J86" s="27" t="inlineStr">
+        <is>
+          <t>decimal ratio</t>
+        </is>
+      </c>
+      <c r="K86" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L86" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M86" s="27" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00459</t>
+        </is>
+      </c>
+      <c r="B87" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C87" s="27" t="inlineStr">
+        <is>
+          <t>Board operating outlook</t>
+        </is>
+      </c>
+      <c r="D87" s="27" t="inlineStr">
+        <is>
+          <t>Controls</t>
+        </is>
+      </c>
+      <c r="E87" s="27" t="inlineStr">
+        <is>
+          <t>2026-05 working copy</t>
+        </is>
+      </c>
+      <c r="F87" s="27" t="inlineStr">
+        <is>
+          <t>Approved case</t>
+        </is>
+      </c>
+      <c r="G87" s="27" t="inlineStr">
+        <is>
+          <t>Forecast opex</t>
+        </is>
+      </c>
+      <c r="H87" s="44" t="n">
+        <v>1113000</v>
+      </c>
+      <c r="I87" s="27" t="inlineStr"/>
+      <c r="J87" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K87" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L87" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M87" s="27" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00460</t>
+        </is>
+      </c>
+      <c r="B88" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C88" s="27" t="inlineStr">
+        <is>
+          <t>Board risk outlook</t>
+        </is>
+      </c>
+      <c r="D88" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E88" s="27" t="inlineStr">
+        <is>
+          <t>Downside</t>
+        </is>
+      </c>
+      <c r="F88" s="27" t="inlineStr">
+        <is>
+          <t>Management stretch</t>
+        </is>
+      </c>
+      <c r="G88" s="27" t="inlineStr">
+        <is>
+          <t>Revolver balance</t>
+        </is>
+      </c>
+      <c r="H88" s="44" t="n">
+        <v>4738000</v>
+      </c>
+      <c r="I88" s="27" t="inlineStr"/>
+      <c r="J88" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K88" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L88" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M88" s="27" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00461</t>
+        </is>
+      </c>
+      <c r="B89" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C89" s="27" t="inlineStr">
+        <is>
+          <t>Board strategic priorities</t>
+        </is>
+      </c>
+      <c r="D89" s="27" t="inlineStr">
+        <is>
+          <t>Service technician hiring</t>
+        </is>
+      </c>
+      <c r="E89" s="27" t="inlineStr">
+        <is>
+          <t>2026-05 working copy</t>
+        </is>
+      </c>
+      <c r="F89" s="27" t="inlineStr">
+        <is>
+          <t>Approved case</t>
+        </is>
+      </c>
+      <c r="G89" s="27" t="inlineStr">
+        <is>
+          <t>Realization probability</t>
+        </is>
+      </c>
+      <c r="H89" s="44" t="n">
+        <v>0.728</v>
+      </c>
+      <c r="I89" s="27" t="inlineStr"/>
+      <c r="J89" s="27" t="inlineStr">
+        <is>
+          <t>decimal ratio</t>
+        </is>
+      </c>
+      <c r="K89" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L89" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M89" s="27" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00462</t>
+        </is>
+      </c>
+      <c r="B90" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C90" s="27" t="inlineStr">
+        <is>
+          <t>Board presentation controls</t>
+        </is>
+      </c>
+      <c r="D90" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E90" s="27" t="inlineStr">
+        <is>
+          <t>FY26</t>
+        </is>
+      </c>
+      <c r="F90" s="27" t="inlineStr">
+        <is>
+          <t>Management stretch</t>
+        </is>
+      </c>
+      <c r="G90" s="27" t="inlineStr">
+        <is>
+          <t>Maximum leverage</t>
+        </is>
+      </c>
+      <c r="H90" s="44" t="n">
+        <v>2.625</v>
+      </c>
+      <c r="I90" s="27" t="inlineStr"/>
+      <c r="J90" s="27" t="inlineStr">
+        <is>
+          <t>multiple</t>
+        </is>
+      </c>
+      <c r="K90" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L90" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M90" s="27" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00463</t>
+        </is>
+      </c>
+      <c r="B91" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C91" s="27" t="inlineStr">
+        <is>
+          <t>Board operating outlook</t>
+        </is>
+      </c>
+      <c r="D91" s="27" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="E91" s="27" t="inlineStr">
+        <is>
+          <t>2026-05 working copy</t>
+        </is>
+      </c>
+      <c r="F91" s="27" t="inlineStr">
+        <is>
+          <t>Approved case</t>
+        </is>
+      </c>
+      <c r="G91" s="27" t="inlineStr">
+        <is>
+          <t>Forecast opex</t>
+        </is>
+      </c>
+      <c r="H91" s="44" t="n">
+        <v>1905500</v>
+      </c>
+      <c r="I91" s="27" t="inlineStr"/>
+      <c r="J91" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K91" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L91" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M91" s="27" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00464</t>
+        </is>
+      </c>
+      <c r="B92" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C92" s="27" t="inlineStr">
+        <is>
+          <t>Board operating outlook</t>
+        </is>
+      </c>
+      <c r="D92" s="27" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E92" s="27" t="inlineStr">
+        <is>
+          <t>FY26</t>
+        </is>
+      </c>
+      <c r="F92" s="27" t="inlineStr">
+        <is>
+          <t>Management stretch</t>
+        </is>
+      </c>
+      <c r="G92" s="27" t="inlineStr">
+        <is>
+          <t>Plan opex</t>
+        </is>
+      </c>
+      <c r="H92" s="44" t="n">
+        <v>2059200</v>
+      </c>
+      <c r="I92" s="27" t="inlineStr"/>
+      <c r="J92" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K92" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L92" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M92" s="27" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00465</t>
+        </is>
+      </c>
+      <c r="B93" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C93" s="27" t="inlineStr">
+        <is>
+          <t>Board risk outlook</t>
+        </is>
+      </c>
+      <c r="D93" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E93" s="27" t="inlineStr">
+        <is>
+          <t>2026-05 working copy</t>
+        </is>
+      </c>
+      <c r="F93" s="27" t="inlineStr">
+        <is>
+          <t>Approved case</t>
+        </is>
+      </c>
+      <c r="G93" s="27" t="inlineStr">
+        <is>
+          <t>Covenant EBITDA</t>
+        </is>
+      </c>
+      <c r="H93" s="44" t="n">
+        <v>5796000</v>
+      </c>
+      <c r="I93" s="27" t="inlineStr"/>
+      <c r="J93" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K93" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L93" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M93" s="27" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00466</t>
+        </is>
+      </c>
+      <c r="B94" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C94" s="27" t="inlineStr">
+        <is>
+          <t>Board risk outlook</t>
+        </is>
+      </c>
+      <c r="D94" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E94" s="27" t="inlineStr">
+        <is>
+          <t>Severe</t>
+        </is>
+      </c>
+      <c r="F94" s="27" t="inlineStr">
+        <is>
+          <t>Management stretch</t>
+        </is>
+      </c>
+      <c r="G94" s="27" t="inlineStr">
+        <is>
+          <t>Ending cash before financing</t>
+        </is>
+      </c>
+      <c r="H94" s="44" t="n">
+        <v>844.6</v>
+      </c>
+      <c r="I94" s="27" t="inlineStr"/>
+      <c r="J94" s="27" t="inlineStr">
+        <is>
+          <t>USD thousands</t>
+        </is>
+      </c>
+      <c r="K94" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L94" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M94" s="27" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00484</t>
+        </is>
+      </c>
+      <c r="B95" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C95" s="27" t="inlineStr">
+        <is>
+          <t>Board decision portfolio</t>
+        </is>
+      </c>
+      <c r="D95" s="27" t="inlineStr">
+        <is>
+          <t>Procurement program</t>
+        </is>
+      </c>
+      <c r="E95" s="27" t="inlineStr">
+        <is>
+          <t>2026-05 working copy</t>
+        </is>
+      </c>
+      <c r="F95" s="27" t="inlineStr">
+        <is>
+          <t>Approved case</t>
+        </is>
+      </c>
+      <c r="G95" s="27" t="inlineStr">
+        <is>
+          <t>Cash investment</t>
+        </is>
+      </c>
+      <c r="H95" s="44" t="n">
+        <v>432600</v>
+      </c>
+      <c r="I95" s="27" t="inlineStr"/>
+      <c r="J95" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K95" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L95" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M95" s="27" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00485</t>
+        </is>
+      </c>
+      <c r="B96" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C96" s="27" t="inlineStr">
+        <is>
+          <t>Board decision portfolio</t>
+        </is>
+      </c>
+      <c r="D96" s="27" t="inlineStr">
+        <is>
+          <t>Pioneer acquisition</t>
+        </is>
+      </c>
+      <c r="E96" s="27" t="inlineStr">
+        <is>
+          <t>FY27</t>
+        </is>
+      </c>
+      <c r="F96" s="27" t="inlineStr">
+        <is>
+          <t>Management stretch</t>
+        </is>
+      </c>
+      <c r="G96" s="27" t="inlineStr">
+        <is>
+          <t>Severe benefit factor</t>
+        </is>
+      </c>
+      <c r="H96" s="44" t="n">
+        <v>0.468</v>
+      </c>
+      <c r="I96" s="27" t="inlineStr"/>
+      <c r="J96" s="27" t="inlineStr">
+        <is>
+          <t>decimal ratio</t>
+        </is>
+      </c>
+      <c r="K96" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L96" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M96" s="27" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00486</t>
+        </is>
+      </c>
+      <c r="B97" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C97" s="27" t="inlineStr">
+        <is>
+          <t>Board decision portfolio</t>
+        </is>
+      </c>
+      <c r="D97" s="27" t="inlineStr">
+        <is>
+          <t>Service technician hiring</t>
+        </is>
+      </c>
+      <c r="E97" s="27" t="inlineStr">
+        <is>
+          <t>2026-05 working copy</t>
+        </is>
+      </c>
+      <c r="F97" s="27" t="inlineStr">
+        <is>
+          <t>Approved case</t>
+        </is>
+      </c>
+      <c r="G97" s="27" t="inlineStr">
+        <is>
+          <t>Severe benefit factor</t>
+        </is>
+      </c>
+      <c r="H97" s="44" t="n">
+        <v>0.6825000000000001</v>
+      </c>
+      <c r="I97" s="27" t="inlineStr"/>
+      <c r="J97" s="27" t="inlineStr">
+        <is>
+          <t>decimal ratio</t>
+        </is>
+      </c>
+      <c r="K97" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L97" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M97" s="27" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00487</t>
+        </is>
+      </c>
+      <c r="B98" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C98" s="27" t="inlineStr">
+        <is>
+          <t>Board decision portfolio policy</t>
+        </is>
+      </c>
+      <c r="D98" s="27" t="inlineStr">
+        <is>
+          <t>Alder Ridge</t>
+        </is>
+      </c>
+      <c r="E98" s="27" t="inlineStr">
+        <is>
+          <t>FY27</t>
+        </is>
+      </c>
+      <c r="F98" s="27" t="inlineStr">
+        <is>
+          <t>Management stretch</t>
+        </is>
+      </c>
+      <c r="G98" s="27" t="inlineStr">
+        <is>
+          <t>Severe EBITDA cash conversion</t>
+        </is>
+      </c>
+      <c r="H98" s="44" t="n">
+        <v>0.721</v>
+      </c>
+      <c r="I98" s="27" t="inlineStr"/>
+      <c r="J98" s="27" t="inlineStr">
+        <is>
+          <t>decimal ratio</t>
+        </is>
+      </c>
+      <c r="K98" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L98" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M98" s="27" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00488</t>
+        </is>
+      </c>
+      <c r="B99" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C99" s="27" t="inlineStr">
+        <is>
+          <t>Board decision portfolio</t>
+        </is>
+      </c>
+      <c r="D99" s="27" t="inlineStr">
+        <is>
+          <t>Pioneer acquisition</t>
+        </is>
+      </c>
+      <c r="E99" s="27" t="inlineStr">
+        <is>
+          <t>2026-05 working copy</t>
+        </is>
+      </c>
+      <c r="F99" s="27" t="inlineStr">
+        <is>
+          <t>Approved case</t>
+        </is>
+      </c>
+      <c r="G99" s="27" t="inlineStr">
+        <is>
+          <t>Cash investment</t>
+        </is>
+      </c>
+      <c r="H99" s="44" t="n">
+        <v>1196000</v>
+      </c>
+      <c r="I99" s="27" t="inlineStr"/>
+      <c r="J99" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K99" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L99" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M99" s="27" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="36" t="inlineStr">
+        <is>
+          <t>RPT-00489</t>
+        </is>
+      </c>
+      <c r="B100" s="27" t="inlineStr">
+        <is>
+          <t>Create the CFO strategic-finance board deck</t>
+        </is>
+      </c>
+      <c r="C100" s="27" t="inlineStr">
+        <is>
+          <t>Board decision portfolio</t>
+        </is>
+      </c>
+      <c r="D100" s="27" t="inlineStr">
+        <is>
+          <t>Service technician hiring</t>
+        </is>
+      </c>
+      <c r="E100" s="27" t="inlineStr">
+        <is>
+          <t>FY27</t>
+        </is>
+      </c>
+      <c r="F100" s="27" t="inlineStr">
+        <is>
+          <t>Management stretch</t>
+        </is>
+      </c>
+      <c r="G100" s="27" t="inlineStr">
+        <is>
+          <t>Cash investment</t>
+        </is>
+      </c>
+      <c r="H100" s="44" t="n">
+        <v>640500</v>
+      </c>
+      <c r="I100" s="27" t="inlineStr"/>
+      <c r="J100" s="27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K100" s="27" t="inlineStr">
+        <is>
+          <t>Earlier management working export</t>
+        </is>
+      </c>
+      <c r="L100" s="45" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="M100" s="27" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M82"/>
+  <autoFilter ref="A4:M100"/>
   <mergeCells count="2">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>

</xml_diff>